<commit_message>
feat: ship Sprache 1.33 UX and practice upgrades
</commit_message>
<xml_diff>
--- a/apps/client/assets/templates/Sprache-easy-import-template.xlsx
+++ b/apps/client/assets/templates/Sprache-easy-import-template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="간편 업로드" sheetId="1" r:id="Rcd3af7612f914859"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작성 안내" sheetId="2" r:id="R898046286d8b40ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="언어키 참고" sheetId="3" r:id="Re253d7ab66844e8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="간편 업로드" sheetId="1" r:id="R0af249308f5c4281"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작성 안내" sheetId="2" r:id="R52016d7b2bf94424"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="언어키 참고" sheetId="3" r:id="R90a42fe0dfb94411"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -60,7 +60,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="37">
+  <x:fills count="43">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -240,6 +240,36 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF4F7F9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2F7F7A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8FBFC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2F7F7A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8FBFC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2F7F7A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8FBFC"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -334,7 +364,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="146">
+  <x:cellXfs count="158">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -656,6 +686,32 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="37" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="37" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="37" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="38" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="38" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="39" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="40" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="41" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="42" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -877,6 +933,7 @@
     <x:col min="16" max="16" width="23" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="24" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="22" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="39" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
@@ -978,6 +1035,9 @@
       <x:c r="R3" s="49" t="str">
         <x:v>distribution_key</x:v>
       </x:c>
+      <x:c r="S3" s="156" t="str">
+        <x:v>id</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
       <x:c r="A4" s="19" t="str">
@@ -1030,6 +1090,7 @@
       <x:c r="R4" s="52" t="str">
         <x:v>lang:en</x:v>
       </x:c>
+      <x:c r="S4" s="157"/>
     </x:row>
     <x:row r="5" ht="38" customHeight="1">
       <x:c r="A5" s="19" t="str">
@@ -1072,6 +1133,7 @@
       <x:c r="R5" s="52" t="str">
         <x:v>lang:en</x:v>
       </x:c>
+      <x:c r="S5" s="157"/>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
       <x:c r="A6" s="19" t="str">
@@ -1122,6 +1184,7 @@
       <x:c r="R6" s="52" t="str">
         <x:v>lang:ja</x:v>
       </x:c>
+      <x:c r="S6" s="157"/>
     </x:row>
     <x:row r="7" ht="38" customHeight="1">
       <x:c r="A7" s="19" t="str">
@@ -1172,6 +1235,7 @@
       <x:c r="R7" s="52" t="str">
         <x:v>lang:de</x:v>
       </x:c>
+      <x:c r="S7" s="157"/>
     </x:row>
     <x:row r="8" ht="38" customHeight="1">
       <x:c r="A8" s="19" t="str">
@@ -1222,6 +1286,7 @@
       <x:c r="R8" s="52" t="str">
         <x:v>lang:fr</x:v>
       </x:c>
+      <x:c r="S8" s="157"/>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
       <x:c r="A9" s="19" t="str">
@@ -1272,6 +1337,7 @@
       <x:c r="R9" s="52" t="str">
         <x:v>lang:es</x:v>
       </x:c>
+      <x:c r="S9" s="157"/>
     </x:row>
     <x:row r="10" ht="38" customHeight="1">
       <x:c r="A10" s="19" t="str">
@@ -1322,6 +1388,7 @@
       <x:c r="R10" s="52" t="str">
         <x:v>lang:zh-hans</x:v>
       </x:c>
+      <x:c r="S10" s="157"/>
     </x:row>
     <x:row r="11" ht="38" customHeight="1">
       <x:c r="A11" s="19" t="str">
@@ -1334,27 +1401,29 @@
         <x:v>OPS</x:v>
       </x:c>
       <x:c r="D11" s="20" t="str">
-        <x:v>출루율과 장타율의 합</x:v>
+        <x:v>출루율과 장타율을 더한 공격 지표</x:v>
       </x:c>
       <x:c r="E11" s="20" t="str">
         <x:v>타격 지표</x:v>
       </x:c>
       <x:c r="F11" s="18" t="str">
-        <x:v>noun</x:v>
-      </x:c>
-      <x:c r="G11" s="18" t="str"/>
+        <x:v>other</x:v>
+      </x:c>
+      <x:c r="G11" s="18" t="str">
+        <x:v>출루율 더하기 장타율|On-base Plus Slugging</x:v>
+      </x:c>
       <x:c r="H11" s="18" t="str">
-        <x:v>OPS가 0.900을 넘었다.</x:v>
+        <x:v>OPS는 출루율과 장타율을 더해 계산한다.</x:v>
       </x:c>
       <x:c r="I11" s="18" t="str">
-        <x:v>좋은 공격력을 보여 줬다.</x:v>
+        <x:v>출루율과 장타율의 합으로 계산하는 공격 지표이다.</x:v>
       </x:c>
       <x:c r="J11" s="18" t="str">
-        <x:v>OPS가|0.900을|넘었다.</x:v>
+        <x:v>OPS는|출루율과|장타율을|더해|계산한다.</x:v>
       </x:c>
       <x:c r="K11" s="18" t="str"/>
       <x:c r="L11" s="18" t="str">
-        <x:v>야구|기록</x:v>
+        <x:v>야구|기초 지표</x:v>
       </x:c>
       <x:c r="M11" s="21" t="str">
         <x:v>기초</x:v>
@@ -1370,6 +1439,9 @@
       <x:c r="R11" s="52" t="str">
         <x:v>baseball-core</x:v>
       </x:c>
+      <x:c r="S11" s="157" t="str">
+        <x:v>1c6b1541-b797-56aa-8255-5767db996318</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="38" customHeight="1">
       <x:c r="A12" s="19" t="str">
@@ -1382,15 +1454,17 @@
         <x:v>OPS</x:v>
       </x:c>
       <x:c r="D12" s="20" t="str">
-        <x:v>타자의 공격력을 나타내는 지표</x:v>
+        <x:v>출루율과 장타율의 합</x:v>
       </x:c>
       <x:c r="E12" s="20" t="str">
         <x:v>이번 주 암기</x:v>
       </x:c>
       <x:c r="F12" s="18" t="str">
-        <x:v>noun</x:v>
-      </x:c>
-      <x:c r="G12" s="18" t="str"/>
+        <x:v>other</x:v>
+      </x:c>
+      <x:c r="G12" s="18" t="str">
+        <x:v>타자의 공격력을 나타내는 지표</x:v>
+      </x:c>
       <x:c r="H12" s="18" t="str"/>
       <x:c r="I12" s="18" t="str"/>
       <x:c r="J12" s="18" t="str"/>
@@ -1412,6 +1486,7 @@
       <x:c r="R12" s="52" t="str">
         <x:v>baseball-core</x:v>
       </x:c>
+      <x:c r="S12" s="157"/>
     </x:row>
     <x:row r="13" ht="38" customHeight="1">
       <x:c r="A13" s="19" t="str">
@@ -1454,11 +1529,12 @@
       <x:c r="R13" s="52" t="str">
         <x:v>lang:en</x:v>
       </x:c>
+      <x:c r="S13" s="157"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:Q1"/>
-    <x:mergeCell ref="A2:Q2"/>
+    <x:mergeCell ref="A1:S1"/>
+    <x:mergeCell ref="A2:S2"/>
   </x:mergeCells>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="A4:A503">
@@ -1726,6 +1802,20 @@
         <x:v>general:baseball</x:v>
       </x:c>
     </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>선택</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>비우면 자동 생성. 번들 자료는 최초 UUID를 계속 유지</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>f64d5def-2065-5768-aeb0-8374e6a201ed</x:v>
+      </x:c>
+    </x:row>
     <x:row r="21">
       <x:c r="A21" s="27" t="str">
         <x:v>가장 중요한 동작</x:v>

</xml_diff>